<commit_message>
ADD: data for april
</commit_message>
<xml_diff>
--- a/transport/transport_data.xlsx
+++ b/transport/transport_data.xlsx
@@ -407,7 +407,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>МАРШРУТ_СНИМКА</t>
+          <t>БРОЙ_ОБЕКТИ</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -2098,11 +2098,6 @@
           <t>Варна-Суворово-Варна</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>{'name': 'viber_image_2026-02-06_17-32-49-760.jpg', 'size': 185211, 'type': 'file', 'upload_time': '2026-02-06T15:33:22.822+00:00', 'url': 'https://cloud.seatable.io/workspace/73766/asset/9ebe8e8a-2c5f-44c3-afdf-b98ab8a88929/external-apps/files/2026-02/viber_image_2026-02-06_17-32-49-760.jpg'}</t>
-        </is>
-      </c>
       <c r="F20" t="inlineStr">
         <is>
           <t>"СИ-ТРАНС БЪЛГАРИЯ"  ЕООД</t>
@@ -5865,10 +5860,10 @@
         <v>38000</v>
       </c>
       <c r="L63" s="2" t="n">
-        <v>485</v>
+        <v>535</v>
       </c>
       <c r="M63" s="3" t="n">
-        <v>12.76315789473684</v>
+        <v>14.07894736842105</v>
       </c>
       <c r="O63" t="inlineStr">
         <is>
@@ -5885,11 +5880,11 @@
       </c>
       <c r="V63" t="inlineStr">
         <is>
-          <t>Plamen Svetoslavov</t>
+          <t>Vesela Nikolova</t>
         </is>
       </c>
       <c r="W63" s="4" t="n">
-        <v>46113.78197206018</v>
+        <v>46126.42932174769</v>
       </c>
       <c r="X63" t="inlineStr">
         <is>
@@ -6572,10 +6567,10 @@
         <v>31500</v>
       </c>
       <c r="L71" s="2" t="n">
-        <v>430</v>
+        <v>452</v>
       </c>
       <c r="M71" s="3" t="n">
-        <v>13.65079365079365</v>
+        <v>14.34920634920635</v>
       </c>
       <c r="O71" t="inlineStr">
         <is>
@@ -6597,11 +6592,11 @@
       </c>
       <c r="V71" t="inlineStr">
         <is>
-          <t>Plamen Svetoslavov</t>
+          <t>Vesela Nikolova</t>
         </is>
       </c>
       <c r="W71" s="4" t="n">
-        <v>46113.78201332176</v>
+        <v>46126.4276888426</v>
       </c>
       <c r="X71" t="inlineStr">
         <is>
@@ -8708,6 +8703,3060 @@
       <c r="Z94" t="inlineStr">
         <is>
           <t>01</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="19.2" customHeight="1">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>20260402-0001</t>
+        </is>
+      </c>
+      <c r="B95" s="1" t="n">
+        <v>46114</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Варна-Каварна-Добрич-Енево-Провадия-Дългопол-Варна</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>CB2201CC</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>P2849EE</t>
+        </is>
+      </c>
+      <c r="J95" s="2" t="n">
+        <v>340</v>
+      </c>
+      <c r="K95" s="2" t="n">
+        <v>33000</v>
+      </c>
+      <c r="L95" s="2" t="n">
+        <v>408</v>
+      </c>
+      <c r="M95" s="3" t="n">
+        <v>12.36363636363636</v>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T95" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U95" s="4" t="n">
+        <v>46114.4417537037</v>
+      </c>
+      <c r="V95" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W95" s="4" t="n">
+        <v>46119.59090974537</v>
+      </c>
+      <c r="X95" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y95" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z95" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="19.2" customHeight="1">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>20260402-0002</t>
+        </is>
+      </c>
+      <c r="B96" s="1" t="n">
+        <v>46113</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Варна-Бяла-Енево-Тервел-Карапелит-Добрич-Ботево-Варна</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>CB2201CC</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>P2849EE</t>
+        </is>
+      </c>
+      <c r="J96" s="2" t="n">
+        <v>540</v>
+      </c>
+      <c r="K96" s="2" t="n">
+        <v>32500</v>
+      </c>
+      <c r="L96" s="2" t="n">
+        <v>648</v>
+      </c>
+      <c r="M96" s="3" t="n">
+        <v>19.93846153846154</v>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T96" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U96" s="4" t="n">
+        <v>46114.44175608797</v>
+      </c>
+      <c r="V96" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W96" s="4" t="n">
+        <v>46119.59081111111</v>
+      </c>
+      <c r="X96" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y96" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z96" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="19.2" customHeight="1">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>20260402-0003</t>
+        </is>
+      </c>
+      <c r="B97" s="1" t="n">
+        <v>46113</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>ОФИС СОФИЯ</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Русе-Бяла-Плевен-Айтос-Поморие-Русе</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>ПАВЕЛ СТЕФАНОВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Р9581МА</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Р4961ЕЕ</t>
+        </is>
+      </c>
+      <c r="J97" s="2" t="n">
+        <v>870</v>
+      </c>
+      <c r="K97" s="2" t="n">
+        <v>39900</v>
+      </c>
+      <c r="L97" s="2" t="n">
+        <v>1044</v>
+      </c>
+      <c r="M97" s="3" t="n">
+        <v>26.16541353383458</v>
+      </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T97" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U97" s="4" t="n">
+        <v>46114.45008017361</v>
+      </c>
+      <c r="V97" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W97" s="4" t="n">
+        <v>46119.59068777777</v>
+      </c>
+      <c r="X97" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y97" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z97" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="19.2" customHeight="1">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>20260402-0004</t>
+        </is>
+      </c>
+      <c r="B98" s="1" t="n">
+        <v>46114</v>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Русе-Бяла-Орешец-Берковица-Враца</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>ДАНИЕЛ ПЕНЧЕВ ПЕНЧЕВ</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Р7826КН</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Р2530ЕЕ</t>
+        </is>
+      </c>
+      <c r="J98" s="2" t="n">
+        <v>470</v>
+      </c>
+      <c r="K98" s="2" t="n">
+        <v>27000</v>
+      </c>
+      <c r="L98" s="2" t="n">
+        <v>564</v>
+      </c>
+      <c r="M98" s="3" t="n">
+        <v>20.88888888888889</v>
+      </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T98" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U98" s="4" t="n">
+        <v>46114.45399453703</v>
+      </c>
+      <c r="V98" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W98" s="4" t="n">
+        <v>46119.59059599537</v>
+      </c>
+      <c r="X98" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y98" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z98" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="19.2" customHeight="1">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>20260407-0001</t>
+        </is>
+      </c>
+      <c r="B99" s="1" t="n">
+        <v>46118</v>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Варна-Добрич-Варна</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>ТРАНС ОЙЛ ЕООД</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>ДИАН СТОЯНОВ АЛЕКСАНДРОВ</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>B7902TM</t>
+        </is>
+      </c>
+      <c r="J99" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="K99" s="2" t="n">
+        <v>10000</v>
+      </c>
+      <c r="L99" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="M99" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T99" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U99" s="4" t="n">
+        <v>46119.58348922454</v>
+      </c>
+      <c r="V99" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W99" s="4" t="n">
+        <v>46119.59397283565</v>
+      </c>
+      <c r="X99" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y99" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z99" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="19.2" customHeight="1">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>20260407-0002</t>
+        </is>
+      </c>
+      <c r="B100" s="1" t="n">
+        <v>46115</v>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>варна-Чефо-Добрич-варна</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>CB2201CC</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>P2849EE</t>
+        </is>
+      </c>
+      <c r="J100" s="2" t="n">
+        <v>130</v>
+      </c>
+      <c r="K100" s="2" t="n">
+        <v>30000</v>
+      </c>
+      <c r="L100" s="2" t="n">
+        <v>156</v>
+      </c>
+      <c r="M100" s="3" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T100" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U100" s="4" t="n">
+        <v>46119.58349258102</v>
+      </c>
+      <c r="V100" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W100" s="4" t="n">
+        <v>46119.59046303241</v>
+      </c>
+      <c r="X100" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y100" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z100" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="19.2" customHeight="1">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>20260407-0003</t>
+        </is>
+      </c>
+      <c r="B101" s="1" t="n">
+        <v>46118</v>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Варна-Повеляново-Калиманци-Любен Каравелово - Вълчи дол - Сенокос- Каварна-Варна</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>CB2201CC</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>P2849EE</t>
+        </is>
+      </c>
+      <c r="J101" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="K101" s="2" t="n">
+        <v>41000</v>
+      </c>
+      <c r="L101" s="2" t="n">
+        <v>360</v>
+      </c>
+      <c r="M101" s="3" t="n">
+        <v>8.780487804878049</v>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T101" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U101" s="4" t="n">
+        <v>46119.59406583333</v>
+      </c>
+      <c r="V101" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W101" s="4" t="n">
+        <v>46119.59755049769</v>
+      </c>
+      <c r="X101" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y101" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z101" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="19.2" customHeight="1">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>20260407-0004</t>
+        </is>
+      </c>
+      <c r="B102" s="1" t="n">
+        <v>46119</v>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Русе-Тервел-Добрич-Стожер-Ушинци-Русе</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>ПАВЕЛ СТЕФАНОВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Р9581МА</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>Р4961ЕЕ</t>
+        </is>
+      </c>
+      <c r="J102" s="2" t="n">
+        <v>440</v>
+      </c>
+      <c r="K102" s="2" t="n">
+        <v>34500</v>
+      </c>
+      <c r="L102" s="2" t="n">
+        <v>528</v>
+      </c>
+      <c r="M102" s="3" t="n">
+        <v>15.30434782608696</v>
+      </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T102" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U102" s="4" t="n">
+        <v>46119.59664443287</v>
+      </c>
+      <c r="V102" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W102" s="4" t="n">
+        <v>46119.59941574074</v>
+      </c>
+      <c r="X102" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y102" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z102" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="19.2" customHeight="1">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>20260407-0005</t>
+        </is>
+      </c>
+      <c r="B103" s="1" t="n">
+        <v>46119</v>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Варна-Девня-Добрич-Ген Колево-Ген. Тошево - Каварна - Варна</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>CB2201CC</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>P2849EE</t>
+        </is>
+      </c>
+      <c r="J103" s="2" t="n">
+        <v>230</v>
+      </c>
+      <c r="K103" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="L103" s="2" t="n">
+        <v>276</v>
+      </c>
+      <c r="M103" s="3" t="n">
+        <v>8.625</v>
+      </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T103" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U103" s="4" t="n">
+        <v>46119.59958134259</v>
+      </c>
+      <c r="V103" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W103" s="4" t="n">
+        <v>46119.60275851852</v>
+      </c>
+      <c r="X103" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y103" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z103" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="19.2" customHeight="1">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>20260407-0006</t>
+        </is>
+      </c>
+      <c r="B104" s="1" t="n">
+        <v>46119</v>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Варна-Добрич-Карапелит-Жегларци-Варна</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>CB2201CC</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>P2849EE</t>
+        </is>
+      </c>
+      <c r="J104" s="2" t="n">
+        <v>260</v>
+      </c>
+      <c r="K104" s="2" t="n">
+        <v>30800</v>
+      </c>
+      <c r="L104" s="2" t="n">
+        <v>312</v>
+      </c>
+      <c r="M104" s="3" t="n">
+        <v>10.12987012987013</v>
+      </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T104" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U104" s="4" t="n">
+        <v>46119.60286013889</v>
+      </c>
+      <c r="V104" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W104" s="4" t="n">
+        <v>46119.60561114583</v>
+      </c>
+      <c r="X104" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y104" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z104" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="19.2" customHeight="1">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>20260407-0007</t>
+        </is>
+      </c>
+      <c r="B105" s="1" t="n">
+        <v>46120</v>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Варна-Бяла-Тервел-Нова Камена-Варна</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>CB2201CC</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>P2849EE</t>
+        </is>
+      </c>
+      <c r="J105" s="2" t="n">
+        <v>510</v>
+      </c>
+      <c r="K105" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="L105" s="2" t="n">
+        <v>612</v>
+      </c>
+      <c r="M105" s="3" t="n">
+        <v>19.125</v>
+      </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T105" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U105" s="4" t="n">
+        <v>46119.60641738426</v>
+      </c>
+      <c r="V105" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W105" s="4" t="n">
+        <v>46121.37460918981</v>
+      </c>
+      <c r="X105" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y105" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z105" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="19.2" customHeight="1">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>20260407-0008</t>
+        </is>
+      </c>
+      <c r="B106" s="1" t="n">
+        <v>46121</v>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Варна-Бяла-Добрич-Каварна-Варна</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>CB2201CC</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>P2849EE</t>
+        </is>
+      </c>
+      <c r="J106" s="2" t="n">
+        <v>550</v>
+      </c>
+      <c r="K106" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="L106" s="2" t="n">
+        <v>660</v>
+      </c>
+      <c r="M106" s="3" t="n">
+        <v>20.625</v>
+      </c>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T106" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U106" s="4" t="n">
+        <v>46119.60840902778</v>
+      </c>
+      <c r="V106" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W106" s="4" t="n">
+        <v>46121.37533226852</v>
+      </c>
+      <c r="X106" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y106" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z106" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="19.2" customHeight="1">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>20260414-0001</t>
+        </is>
+      </c>
+      <c r="B107" s="1" t="n">
+        <v>46120</v>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Русе-Бяла-Търговище-Шумен-Снежина-Русе</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>ПАВЕЛ СТЕФАНОВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Р9581МА</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>Р4961ЕЕ</t>
+        </is>
+      </c>
+      <c r="J107" s="2" t="n">
+        <v>380</v>
+      </c>
+      <c r="K107" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="L107" s="2" t="n">
+        <v>456</v>
+      </c>
+      <c r="M107" s="3" t="n">
+        <v>14.25</v>
+      </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T107" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U107" s="4" t="n">
+        <v>46126.38869865741</v>
+      </c>
+      <c r="V107" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W107" s="4" t="n">
+        <v>46126.39018428241</v>
+      </c>
+      <c r="X107" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y107" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z107" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="19.2" customHeight="1">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>20260414-0002</t>
+        </is>
+      </c>
+      <c r="B108" s="1" t="n">
+        <v>46126</v>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Варна-Русе-Бяла-Девня-Добрич-Каварна-Варна</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>CB2201CC</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>P2849EE</t>
+        </is>
+      </c>
+      <c r="J108" s="2" t="n">
+        <v>600</v>
+      </c>
+      <c r="K108" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="L108" s="2" t="n">
+        <v>720</v>
+      </c>
+      <c r="M108" s="3" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T108" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U108" s="4" t="n">
+        <v>46126.3906471875</v>
+      </c>
+      <c r="V108" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W108" s="4" t="n">
+        <v>46126.39402790509</v>
+      </c>
+      <c r="X108" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y108" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z108" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="19.2" customHeight="1">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>20260414-0003</t>
+        </is>
+      </c>
+      <c r="B109" s="1" t="n">
+        <v>46126</v>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Русе-Бяла-Тервел-Добрич-Русе</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>ДАНИЕЛ ПЕНЧЕВ ПЕНЧЕВ</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Р7826КН</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>Р2530ЕЕ</t>
+        </is>
+      </c>
+      <c r="J109" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="K109" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="L109" s="2" t="n">
+        <v>600</v>
+      </c>
+      <c r="M109" s="3" t="n">
+        <v>18.75</v>
+      </c>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T109" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U109" s="4" t="n">
+        <v>46126.39436719907</v>
+      </c>
+      <c r="V109" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W109" s="4" t="n">
+        <v>46126.39566355324</v>
+      </c>
+      <c r="X109" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y109" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z109" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="19.2" customHeight="1">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>20260424-0001</t>
+        </is>
+      </c>
+      <c r="B110" s="1" t="n">
+        <v>46127</v>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Варна-Бяла-Блъсково-Повеляново-Варна-Стожер-Добрич-Ген.Киселово-Брестак-Есеница-Карапелит-Окорш-Бяла</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>CB2201CC</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>P2849EE</t>
+        </is>
+      </c>
+      <c r="J110" s="2" t="n">
+        <v>800</v>
+      </c>
+      <c r="K110" s="2" t="n">
+        <v>31000</v>
+      </c>
+      <c r="L110" s="2" t="n">
+        <v>960</v>
+      </c>
+      <c r="M110" s="3" t="n">
+        <v>30.96774193548387</v>
+      </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T110" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U110" s="4" t="n">
+        <v>46136.67863891204</v>
+      </c>
+      <c r="V110" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W110" s="4" t="n">
+        <v>46136.68043775463</v>
+      </c>
+      <c r="X110" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y110" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z110" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="19.2" customHeight="1">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>20260424-0002</t>
+        </is>
+      </c>
+      <c r="B111" s="1" t="n">
+        <v>46129</v>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Варна-Бяла-Добрич-Каварна-варна</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>CB2201CC</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>P2849EE</t>
+        </is>
+      </c>
+      <c r="J111" s="2" t="n">
+        <v>550</v>
+      </c>
+      <c r="K111" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="L111" s="2" t="n">
+        <v>660</v>
+      </c>
+      <c r="M111" s="3" t="n">
+        <v>20.625</v>
+      </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T111" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U111" s="4" t="n">
+        <v>46136.68062988426</v>
+      </c>
+      <c r="V111" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W111" s="4" t="n">
+        <v>46136.69066723379</v>
+      </c>
+      <c r="X111" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y111" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z111" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="19.2" customHeight="1">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>20260424-0003</t>
+        </is>
+      </c>
+      <c r="B112" s="1" t="n">
+        <v>46132</v>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Русе-Бяла-Тервел-Русе</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>ПАВЕЛ СТЕФАНОВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>CB2201CC</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>P2849EE</t>
+        </is>
+      </c>
+      <c r="J112" s="2" t="n">
+        <v>420</v>
+      </c>
+      <c r="K112" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="L112" s="2" t="n">
+        <v>504</v>
+      </c>
+      <c r="M112" s="3" t="n">
+        <v>15.75</v>
+      </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T112" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U112" s="4" t="n">
+        <v>46136.69078819444</v>
+      </c>
+      <c r="V112" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W112" s="4" t="n">
+        <v>46136.69432903935</v>
+      </c>
+      <c r="X112" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y112" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z112" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="19.2" customHeight="1">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>20260424-0004</t>
+        </is>
+      </c>
+      <c r="B113" s="1" t="n">
+        <v>46132</v>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Варна-Русе-Бяла-Каварна-Близнаци-Повеляново-Варна</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>Р9581МА</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>Р4961ЕЕ</t>
+        </is>
+      </c>
+      <c r="J113" s="2" t="n">
+        <v>580</v>
+      </c>
+      <c r="K113" s="2" t="n">
+        <v>30000</v>
+      </c>
+      <c r="L113" s="2" t="n">
+        <v>696</v>
+      </c>
+      <c r="M113" s="3" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T113" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U113" s="4" t="n">
+        <v>46136.69437859954</v>
+      </c>
+      <c r="V113" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W113" s="4" t="n">
+        <v>46136.69595549769</v>
+      </c>
+      <c r="X113" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y113" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z113" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="19.2" customHeight="1">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>20260424-0005</t>
+        </is>
+      </c>
+      <c r="B114" s="1" t="n">
+        <v>46133</v>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Варна-Добрич-Варна</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Р9581МА</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>Р4961ЕЕ</t>
+        </is>
+      </c>
+      <c r="J114" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="K114" s="2" t="n">
+        <v>30000</v>
+      </c>
+      <c r="L114" s="2" t="n">
+        <v>600</v>
+      </c>
+      <c r="M114" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T114" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U114" s="4" t="n">
+        <v>46136.69599675926</v>
+      </c>
+      <c r="V114" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W114" s="4" t="n">
+        <v>46136.69708907408</v>
+      </c>
+      <c r="X114" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y114" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z114" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="19.2" customHeight="1">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>20260424-0006</t>
+        </is>
+      </c>
+      <c r="B115" s="1" t="n">
+        <v>46134</v>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Бяла-Ловеч-Павликени-Бяла</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Р9581МА</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Р4961ЕЕ</t>
+        </is>
+      </c>
+      <c r="J115" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="K115" s="2" t="n">
+        <v>30000</v>
+      </c>
+      <c r="L115" s="2" t="n">
+        <v>360</v>
+      </c>
+      <c r="M115" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T115" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U115" s="4" t="n">
+        <v>46136.69714005787</v>
+      </c>
+      <c r="V115" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W115" s="4" t="n">
+        <v>46136.70557487269</v>
+      </c>
+      <c r="X115" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y115" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z115" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="19.2" customHeight="1">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>20260424-0007</t>
+        </is>
+      </c>
+      <c r="B116" s="1" t="n">
+        <v>46135</v>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Варна-Бяла-Тервел-Добрич-Малина-Каварна-Варна</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Р9581МА</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Р4961ЕЕ</t>
+        </is>
+      </c>
+      <c r="J116" s="2" t="n">
+        <v>570</v>
+      </c>
+      <c r="K116" s="2" t="n">
+        <v>30000</v>
+      </c>
+      <c r="L116" s="2" t="n">
+        <v>690</v>
+      </c>
+      <c r="M116" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T116" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U116" s="4" t="n">
+        <v>46136.70620979166</v>
+      </c>
+      <c r="V116" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W116" s="4" t="n">
+        <v>46136.70717837963</v>
+      </c>
+      <c r="X116" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y116" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z116" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="19.2" customHeight="1">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>20260424-0008</t>
+        </is>
+      </c>
+      <c r="B117" s="1" t="n">
+        <v>46136</v>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Варна-Добрич-Повеляново-Варна</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Р9581МА</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>Р4961ЕЕ</t>
+        </is>
+      </c>
+      <c r="J117" s="2" t="n">
+        <v>140</v>
+      </c>
+      <c r="K117" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="L117" s="2" t="n">
+        <v>168</v>
+      </c>
+      <c r="M117" s="3" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T117" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U117" s="4" t="n">
+        <v>46136.7072147338</v>
+      </c>
+      <c r="V117" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W117" s="4" t="n">
+        <v>46136.7084734375</v>
+      </c>
+      <c r="X117" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y117" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z117" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="19.2" customHeight="1">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>20260424-0009</t>
+        </is>
+      </c>
+      <c r="B118" s="1" t="n">
+        <v>46139</v>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Варна-Сл.Бряг-Несебър-НХК-Риш-Нова Бяла Река-Провадия-Енево-Добрич-Варна</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Р9581МА</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>Р4961ЕЕ</t>
+        </is>
+      </c>
+      <c r="J118" s="2" t="n">
+        <v>510</v>
+      </c>
+      <c r="K118" s="2" t="n">
+        <v>42500</v>
+      </c>
+      <c r="L118" s="2" t="n">
+        <v>510</v>
+      </c>
+      <c r="M118" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T118" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U118" s="4" t="n">
+        <v>46136.70855460648</v>
+      </c>
+      <c r="V118" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W118" s="4" t="n">
+        <v>46136.7159302662</v>
+      </c>
+      <c r="X118" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y118" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z118" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="19.2" customHeight="1">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>20260424-0010</t>
+        </is>
+      </c>
+      <c r="B119" s="1" t="n">
+        <v>46139</v>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Русе-тервел-Русе</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>ДАНИЕЛ ПЕНЧЕВ ПЕНЧЕВ</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Р7826КН</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>Р2530ЕЕ</t>
+        </is>
+      </c>
+      <c r="J119" s="2" t="n">
+        <v>330</v>
+      </c>
+      <c r="K119" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="L119" s="2" t="n">
+        <v>330</v>
+      </c>
+      <c r="M119" s="3" t="n">
+        <v>10.3125</v>
+      </c>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T119" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U119" s="4" t="n">
+        <v>46136.71483799769</v>
+      </c>
+      <c r="V119" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W119" s="4" t="n">
+        <v>46136.71601056713</v>
+      </c>
+      <c r="X119" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y119" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z119" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="19.2" customHeight="1">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>20260424-0011</t>
+        </is>
+      </c>
+      <c r="B120" s="1" t="n">
+        <v>46139</v>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Русе-Бяла-Лом-Орешец-Русе</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>ПАВЕЛ СТЕФАНОВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>CB2201CC</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>P2849EE</t>
+        </is>
+      </c>
+      <c r="J120" s="2" t="n">
+        <v>700</v>
+      </c>
+      <c r="K120" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="L120" s="2" t="n">
+        <v>840</v>
+      </c>
+      <c r="M120" s="3" t="n">
+        <v>26.25</v>
+      </c>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T120" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U120" s="4" t="n">
+        <v>46136.71606890046</v>
+      </c>
+      <c r="V120" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W120" s="4" t="n">
+        <v>46136.71730175926</v>
+      </c>
+      <c r="X120" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y120" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z120" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="19.2" customHeight="1">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>20260428-0001</t>
+        </is>
+      </c>
+      <c r="B121" s="1" t="n">
+        <v>46129</v>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>НХК-Каблешково-НХК</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>ДИРОСИ ООД</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>СТАНИСЛАВ ДИМИТРОВ ИВАНОВ</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>А1535ВВ</t>
+        </is>
+      </c>
+      <c r="J121" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="K121" s="2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="L121" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="M121" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T121" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U121" s="4" t="n">
+        <v>46140.64835413195</v>
+      </c>
+      <c r="V121" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W121" s="4" t="n">
+        <v>46140.65173761574</v>
+      </c>
+      <c r="X121" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y121" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z121" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="19.2" customHeight="1">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>20260428-0002</t>
+        </is>
+      </c>
+      <c r="B122" s="1" t="n">
+        <v>46140</v>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>ВАРНА-девня-Варна</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Р9581МА</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>Р4961ЕЕ</t>
+        </is>
+      </c>
+      <c r="J122" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="K122" s="2" t="n">
+        <v>18000</v>
+      </c>
+      <c r="L122" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="M122" s="3" t="n">
+        <v>6.666666666666667</v>
+      </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T122" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U122" s="4" t="n">
+        <v>46140.65242412037</v>
+      </c>
+      <c r="V122" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W122" s="4" t="n">
+        <v>46140.66494774305</v>
+      </c>
+      <c r="X122" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y122" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z122" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="19.2" customHeight="1">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>20260428-0003</t>
+        </is>
+      </c>
+      <c r="B123" s="1" t="n">
+        <v>46140</v>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Варна-Добрич-Варна</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Р9581МА</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>Р4961ЕЕ</t>
+        </is>
+      </c>
+      <c r="J123" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="K123" s="2" t="n">
+        <v>26000</v>
+      </c>
+      <c r="L123" s="2" t="n">
+        <v>144</v>
+      </c>
+      <c r="M123" s="3" t="n">
+        <v>5.538461538461538</v>
+      </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T123" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U123" s="4" t="n">
+        <v>46140.66499206018</v>
+      </c>
+      <c r="V123" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W123" s="4" t="n">
+        <v>46140.66614908565</v>
+      </c>
+      <c r="X123" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y123" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z123" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="19.2" customHeight="1">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>20260428-0004</t>
+        </is>
+      </c>
+      <c r="B124" s="1" t="n">
+        <v>46141</v>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Варна-Долни Чифлик- Невестино- Деветак - НХК</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>Р9581МА</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>Р4961ЕЕ</t>
+        </is>
+      </c>
+      <c r="J124" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="K124" s="2" t="n">
+        <v>14500</v>
+      </c>
+      <c r="L124" s="2" t="n">
+        <v>360</v>
+      </c>
+      <c r="M124" s="3" t="n">
+        <v>24.82758620689655</v>
+      </c>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T124" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U124" s="4" t="n">
+        <v>46140.6661940625</v>
+      </c>
+      <c r="V124" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W124" s="4" t="n">
+        <v>46140.66803032407</v>
+      </c>
+      <c r="X124" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y124" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z124" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="19.2" customHeight="1">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>20260428-0005</t>
+        </is>
+      </c>
+      <c r="B125" s="1" t="n">
+        <v>46142</v>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Варна-Добрич-Русе</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>ДАНИЕЛ ПЕНЧЕВ ПЕНЧЕВ</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Р7826КН</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>Р2530ЕЕ</t>
+        </is>
+      </c>
+      <c r="J125" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="K125" s="2" t="n">
+        <v>23500</v>
+      </c>
+      <c r="L125" s="2" t="n">
+        <v>360</v>
+      </c>
+      <c r="M125" s="3" t="n">
+        <v>15.31914893617021</v>
+      </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T125" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U125" s="4" t="n">
+        <v>46140.66811951389</v>
+      </c>
+      <c r="V125" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W125" s="4" t="n">
+        <v>46142.62504547454</v>
+      </c>
+      <c r="X125" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y125" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z125" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="19.2" customHeight="1">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>20260428-0006</t>
+        </is>
+      </c>
+      <c r="B126" s="1" t="n">
+        <v>46142</v>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>НХК-Пчелник-Повеляново-Варна-Карапелит-Тервел-НХК</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>Р9581МА</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>Р4961ЕЕ</t>
+        </is>
+      </c>
+      <c r="J126" s="2" t="n">
+        <v>370</v>
+      </c>
+      <c r="K126" s="2" t="n">
+        <v>30000</v>
+      </c>
+      <c r="L126" s="2" t="n">
+        <v>444</v>
+      </c>
+      <c r="M126" s="3" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T126" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U126" s="4" t="n">
+        <v>46140.66816375</v>
+      </c>
+      <c r="V126" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W126" s="4" t="n">
+        <v>46140.67040407407</v>
+      </c>
+      <c r="X126" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y126" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z126" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="19.2" customHeight="1">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>20260430-0001</t>
+        </is>
+      </c>
+      <c r="B127" s="1" t="n">
+        <v>46142</v>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Варна-Ботево-Варна</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>Р9581МА</t>
+        </is>
+      </c>
+      <c r="J127" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="K127" s="2" t="n">
+        <v>12000</v>
+      </c>
+      <c r="L127" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="M127" s="3" t="n">
+        <v>7.333333333333333</v>
+      </c>
+      <c r="O127" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T127" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U127" s="4" t="n">
+        <v>46142.62276876158</v>
+      </c>
+      <c r="V127" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W127" s="4" t="n">
+        <v>46142.6237709375</v>
+      </c>
+      <c r="X127" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y127" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="Z127" t="inlineStr">
+        <is>
+          <t>30</t>
         </is>
       </c>
     </row>

</xml_diff>